<commit_message>
Parsing Shareholder Holding Data - Parser.py
</commit_message>
<xml_diff>
--- a/DSE_Company_Details.xlsx
+++ b/DSE_Company_Details.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM2"/>
+  <dimension ref="A1:AS2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,52 +564,82 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>Instrument Type</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>Debut Trading Date</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Instrument Type</t>
-        </is>
-      </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>Listing Year</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Market Category</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Electronic Share</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
           <t>Last AGM held on</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>For the year ended</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Last Div Year</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Last Div Yield</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Cash Dividend</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Bonus Issue (Stock Dividend)</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Last Div Yield</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Right Issue</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Year End</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Share Holding Percentage [as on Jun 30, 2025 (year ended)]</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Share Holding Percentage [as on Feb 28, 2026]</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Share Holding Percentage [as on Mar 31, 2026]</t>
         </is>
       </c>
     </row>
@@ -713,52 +743,82 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
           <t>14 Jun, 2012</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
       <c r="AF2" t="inlineStr">
         <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
           <t>23-11-2025</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Jun 30, 2025</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>3.21</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
         <is>
           <t>40% 2025, 40% 2024, 51% 2023, 46% 2022, 37% 2021, 20% 2020, 16% 2019, 5% 2018, 12% 2017, 10% 2016, 10% 2014, 20% 2013, 20% 2012</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>10% 2015, 15% 2013, 10% 2012</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>3.21</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>30-Jun</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>Sponsor/Director: 0.00 | Govt: 76.93 | Institute: 15.23 | Foreign: 2.07 | Public: 5.77</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>Sponsor/Director: 0.00 | Govt: 76.94 | Institute: 17.22 | Foreign: 0.08 | Public: 5.76</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Sponsor/Director: 0.00 | Govt: 76.94 | Institute: 17.52 | Foreign: 0.07 | Public: 5.47</t>
         </is>
       </c>
     </row>

</xml_diff>